<commit_message>
Report update @ 01-Sep-2025 08:50:11
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -4345,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D74" t="n">
         <v>11</v>
@@ -4369,10 +4369,10 @@
         <v>26</v>
       </c>
       <c r="K74" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L74" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M74" t="n">
         <v>12</v>
@@ -4381,7 +4381,7 @@
         <v>1</v>
       </c>
       <c r="O74" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P74" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
Report update @ 02-Sep-2025 14:28:22
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4390,6 +4390,59 @@
         <v>29</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B75" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Report update @ 04-Sep-2025 22:31:26
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4345,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D74" t="n">
         <v>11</v>
@@ -4369,10 +4369,10 @@
         <v>26</v>
       </c>
       <c r="K74" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L74" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M74" t="n">
         <v>12</v>
@@ -4381,13 +4381,66 @@
         <v>1</v>
       </c>
       <c r="O74" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P74" t="n">
         <v>13</v>
       </c>
       <c r="Q74" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B75" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
+        <v>1</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report update @ 05-Sep-2025 14:51:11
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -4398,37 +4398,37 @@
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N75" t="n">
         <v>0</v>
@@ -4440,7 +4440,7 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report update @ 06-Sep-2025 12:19:25
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -4398,10 +4398,10 @@
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
@@ -4413,16 +4413,16 @@
         <v>1</v>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L75" t="n">
         <v>1</v>
@@ -4440,7 +4440,7 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report update @ 06-Sep-2025 20:34:35
</commit_message>
<xml_diff>
--- a/aircraft/reports/aircraft-type-trends-monthly.xlsx
+++ b/aircraft/reports/aircraft-type-trends-monthly.xlsx
@@ -4398,22 +4398,22 @@
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D75" t="n">
         <v>2</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>2</v>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H75" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
@@ -4422,25 +4422,25 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M75" t="n">
         <v>3</v>
       </c>
       <c r="N75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P75" t="n">
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>